<commit_message>
sửa 1 ít giao diện
</commit_message>
<xml_diff>
--- a/IMEI_IP18-DO-128.xlsx
+++ b/IMEI_IP18-DO-128.xlsx
@@ -19,36 +19,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="2">
   <si>
     <t>IP18-DO-128</t>
   </si>
   <si>
-    <t>359123456789102</t>
-  </si>
-  <si>
-    <t>359123456789103</t>
-  </si>
-  <si>
-    <t>359123456789104</t>
-  </si>
-  <si>
-    <t>359123456789105</t>
-  </si>
-  <si>
-    <t>359123456789106</t>
-  </si>
-  <si>
-    <t>359123456789107</t>
-  </si>
-  <si>
-    <t>359123456789108</t>
-  </si>
-  <si>
-    <t>359123456789109</t>
-  </si>
-  <si>
-    <t>359123456789110</t>
+    <t>IP18-HONG-128</t>
   </si>
 </sst>
 </file>
@@ -84,8 +60,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -366,113 +343,176 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:C10"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="1" width="15.21875" customWidth="1"/>
     <col min="2" max="2" width="27.21875" customWidth="1"/>
     <col min="3" max="3" width="33.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1">
+        <v>1</v>
+      </c>
+      <c r="B1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="1">
         <v>459123456789002</v>
       </c>
-      <c r="C2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>0</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="1">
         <v>459123456789003</v>
       </c>
-      <c r="C3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>0</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="1">
         <v>459123456789004</v>
       </c>
-      <c r="C4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>0</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="1">
         <v>459123456789005</v>
       </c>
-      <c r="C5" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>0</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="1">
         <v>459123456789006</v>
       </c>
-      <c r="C6" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>0</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="1">
         <v>459123456789007</v>
       </c>
-      <c r="C7" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>0</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="1">
         <v>459123456789008</v>
       </c>
-      <c r="C8" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>0</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="1">
         <v>459123456789009</v>
       </c>
-      <c r="C9" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>0</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="1">
         <v>459123456789010</v>
       </c>
-      <c r="C10" t="s">
-        <v>9</v>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="1">
+        <v>359123456789102</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B12" s="1">
+        <v>359123456789103</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>1</v>
+      </c>
+      <c r="B13" s="1">
+        <v>359123456789104</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>1</v>
+      </c>
+      <c r="B14" s="1">
+        <v>359123456789105</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B15" s="1">
+        <v>359123456789106</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>1</v>
+      </c>
+      <c r="B16" s="1">
+        <v>359123456789107</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>1</v>
+      </c>
+      <c r="B17" s="1">
+        <v>359123456789108</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B18" s="1">
+        <v>359123456789109</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>1</v>
+      </c>
+      <c r="B19" s="1">
+        <v>359123456789110</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>1</v>
+      </c>
+      <c r="B20" s="1">
+        <v>359123456789111</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>